<commit_message>
blacklist excel ve json temizlendi
</commit_message>
<xml_diff>
--- a/output/amazon_niche_rapor_2026-03-31.xlsx
+++ b/output/amazon_niche_rapor_2026-03-31.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F188"/>
+  <dimension ref="A1:F167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -3280,23 +3280,23 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>3k oled laptop 16</t>
+          <t>3k taramps amp bass</t>
         </is>
       </c>
       <c r="B102" s="2" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>$1473.99</t>
+          <t>$251.81</t>
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
@@ -3308,23 +3308,23 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>3k taramps amp bass</t>
+          <t>3k watt amp wiring kit ofc</t>
         </is>
       </c>
       <c r="B103" s="2" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>$251.81</t>
+          <t>$79.87</t>
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>46.2%</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -3336,15 +3336,15 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>3k watt amp wiring kit ofc</t>
+          <t>3k bass amp</t>
         </is>
       </c>
       <c r="B104" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>$79.87</t>
+          <t>$205.96</t>
         </is>
       </c>
       <c r="D104" s="2" t="n">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>46.2%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
@@ -3364,23 +3364,23 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>3k bass amp</t>
+          <t>83 inch oled tv samsung</t>
         </is>
       </c>
       <c r="B105" s="2" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>$205.96</t>
+          <t>$2522.85</t>
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
@@ -3392,7 +3392,7 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>83 inch oled tv samsung</t>
+          <t>83 inch oled tv g4</t>
         </is>
       </c>
       <c r="B106" s="2" t="n">
@@ -3400,7 +3400,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>$2522.85</t>
+          <t>$39.99</t>
         </is>
       </c>
       <c r="D106" s="2" t="n">
@@ -3420,23 +3420,23 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>83 inch oled tv g4</t>
+          <t>83 inch oled tv gaming</t>
         </is>
       </c>
       <c r="B107" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>$172.64</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C107" s="2" t="inlineStr">
-        <is>
-          <t>$39.99</t>
-        </is>
-      </c>
-      <c r="D107" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
@@ -3448,23 +3448,23 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>83 inch oled tv gaming</t>
+          <t>3k monitor 240hz</t>
         </is>
       </c>
       <c r="B108" s="2" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>$172.64</t>
+          <t>$338.03</t>
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
@@ -3476,23 +3476,23 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>3k monitor 240hz</t>
+          <t>sprayway stainless steel cleaner</t>
         </is>
       </c>
       <c r="B109" s="2" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>$338.03</t>
+          <t>$17.37</t>
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
@@ -3504,23 +3504,23 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>sprayway stainless steel cleaner</t>
+          <t>66 inch tv</t>
         </is>
       </c>
       <c r="B110" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>$103.12</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C110" s="2" t="inlineStr">
-        <is>
-          <t>$17.37</t>
-        </is>
-      </c>
-      <c r="D110" s="2" t="n">
-        <v>2</v>
-      </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>66.7%</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
@@ -3532,23 +3532,23 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>66 inch tv</t>
+          <t>xxxl stainless steel litter box</t>
         </is>
       </c>
       <c r="B111" s="2" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>$103.12</t>
+          <t>$94.60</t>
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>48.0%</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
@@ -3560,23 +3560,23 @@
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>xxxl stainless steel litter box</t>
+          <t>83 inch oled tv c5</t>
         </is>
       </c>
       <c r="B112" s="2" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>$94.60</t>
+          <t>$108.96</t>
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>48.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
@@ -3588,23 +3588,23 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>83 inch oled tv c5</t>
+          <t>gardening organizer cart</t>
         </is>
       </c>
       <c r="B113" s="2" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>$108.96</t>
+          <t>$72.95</t>
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>47.1%</t>
         </is>
       </c>
       <c r="F113" s="2" t="inlineStr">
@@ -3616,23 +3616,23 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>gardening organizer cart</t>
+          <t>plug in solar panels for homes</t>
         </is>
       </c>
       <c r="B114" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>$72.95</t>
+          <t>$143.94</t>
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>47.1%</t>
+          <t>60.0%</t>
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr">
@@ -3644,23 +3644,23 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>plug in solar panels for homes</t>
+          <t>66 roots journey bible study</t>
         </is>
       </c>
       <c r="B115" s="2" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>$143.94</t>
+          <t>$17.41</t>
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>41.7%</t>
         </is>
       </c>
       <c r="F115" s="2" t="inlineStr">
@@ -3672,23 +3672,23 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>66 roots journey bible study</t>
+          <t>3k amplifier 4 channel</t>
         </is>
       </c>
       <c r="B116" s="2" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>$17.41</t>
+          <t>$181.03</t>
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>41.7%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
@@ -3700,23 +3700,23 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>3k amplifier 4 channel</t>
+          <t>stainless steel litter box sifting</t>
         </is>
       </c>
       <c r="B117" s="2" t="n">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>$181.03</t>
+          <t>$70.33</t>
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>44.1%</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
@@ -3728,23 +3728,23 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>stainless steel litter box sifting</t>
+          <t>3k taramps amp 4 channel</t>
         </is>
       </c>
       <c r="B118" s="2" t="n">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>$70.33</t>
+          <t>$200.81</t>
         </is>
       </c>
       <c r="D118" s="2" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>44.1%</t>
+          <t>46.7%</t>
         </is>
       </c>
       <c r="F118" s="2" t="inlineStr">
@@ -3756,23 +3756,23 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>3k taramps amp 4 channel</t>
+          <t>3k bass amp taramps</t>
         </is>
       </c>
       <c r="B119" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>$200.81</t>
+          <t>$251.94</t>
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>46.7%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">
@@ -3784,19 +3784,19 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>3k bass amp taramps</t>
+          <t>83 oled lg</t>
         </is>
       </c>
       <c r="B120" s="2" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>$251.94</t>
+          <t>$486.18</t>
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
@@ -3812,23 +3812,23 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>83 oled lg</t>
+          <t>2032 battery 2 pack</t>
         </is>
       </c>
       <c r="B121" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>$486.18</t>
+          <t>$29.36</t>
         </is>
       </c>
       <c r="D121" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F121" s="2" t="inlineStr">
@@ -3840,23 +3840,23 @@
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>2032 battery 2 pack</t>
+          <t>66 page bible study guide extra large print</t>
         </is>
       </c>
       <c r="B122" s="2" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>$29.36</t>
+          <t>$19.91</t>
         </is>
       </c>
       <c r="D122" s="2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>43.5%</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
@@ -3868,15 +3868,15 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>66 page bible study guide extra large print</t>
+          <t>kettlebell rack stand only</t>
         </is>
       </c>
       <c r="B123" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>$19.91</t>
+          <t>$63.81</t>
         </is>
       </c>
       <c r="D123" s="2" t="n">
@@ -3884,7 +3884,7 @@
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>43.5%</t>
+          <t>45.5%</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
@@ -3896,23 +3896,23 @@
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>kettlebell rack stand only</t>
+          <t>66 inch tv console</t>
         </is>
       </c>
       <c r="B124" s="2" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>$63.81</t>
+          <t>$118.36</t>
         </is>
       </c>
       <c r="D124" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>44.8%</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
@@ -3924,23 +3924,23 @@
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>66 inch tv console</t>
+          <t>katori titanium cutting board</t>
         </is>
       </c>
       <c r="B125" s="2" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>$118.36</t>
+          <t>$46.81</t>
         </is>
       </c>
       <c r="D125" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>44.8%</t>
+          <t>45.5%</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
@@ -3952,23 +3952,23 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>katori titanium cutting board</t>
+          <t>3k taramps amp 2 ohm</t>
         </is>
       </c>
       <c r="B126" s="2" t="n">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>$46.81</t>
+          <t>$222.78</t>
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
@@ -3980,23 +3980,23 @@
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>3k taramps amp 2 ohm</t>
+          <t>plug in solar panels</t>
         </is>
       </c>
       <c r="B127" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>$147.84</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C127" s="2" t="inlineStr">
-        <is>
-          <t>$222.78</t>
-        </is>
-      </c>
-      <c r="D127" s="2" t="n">
-        <v>6</v>
-      </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>63.6%</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
@@ -4008,23 +4008,23 @@
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>plug in solar panels</t>
+          <t>3k taramps amp 1 ohm</t>
         </is>
       </c>
       <c r="B128" s="2" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>$147.84</t>
+          <t>$195.43</t>
         </is>
       </c>
       <c r="D128" s="2" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>63.6%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
@@ -4036,23 +4036,23 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>3k taramps amp 1 ohm</t>
+          <t>3k taramps amp 4 ohm</t>
         </is>
       </c>
       <c r="B129" s="2" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>$195.43</t>
+          <t>$198.57</t>
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>42.1%</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
@@ -4064,15 +4064,15 @@
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>3k taramps amp 4 ohm</t>
+          <t>3k amp 2 channel</t>
         </is>
       </c>
       <c r="B130" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>$198.57</t>
+          <t>$189.54</t>
         </is>
       </c>
       <c r="D130" s="2" t="n">
@@ -4080,7 +4080,7 @@
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>42.1%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
@@ -4092,23 +4092,23 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>3k amp 2 channel</t>
+          <t>3k amp wiring kit</t>
         </is>
       </c>
       <c r="B131" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>$189.54</t>
+          <t>$47.04</t>
         </is>
       </c>
       <c r="D131" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
@@ -4120,23 +4120,23 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>3k amp wiring kit</t>
+          <t>83 inch oled tvs</t>
         </is>
       </c>
       <c r="B132" s="2" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>$47.04</t>
+          <t>$135.49</t>
         </is>
       </c>
       <c r="D132" s="2" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
@@ -4148,15 +4148,15 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>83 inch oled tvs</t>
+          <t>4.64.6 out of 5 stars(173)300+ bought in past month</t>
         </is>
       </c>
       <c r="B133" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>$135.49</t>
+          <t>$86.99</t>
         </is>
       </c>
       <c r="D133" s="2" t="n">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
@@ -4176,23 +4176,23 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>4.64.6 out of 5 stars(173)300+ bought in past month</t>
+          <t>52 inch ceiling fan with light and remote white</t>
         </is>
       </c>
       <c r="B134" s="2" t="n">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>$86.99</t>
+          <t>$94.67</t>
         </is>
       </c>
       <c r="D134" s="2" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>40.6%</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
@@ -4204,23 +4204,23 @@
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>52 inch ceiling fan with light and remote white</t>
+          <t>52 inch ceiling fan with light and remote downrod</t>
         </is>
       </c>
       <c r="B135" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>$94.67</t>
+          <t>$95.93</t>
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>40.6%</t>
+          <t>42.4%</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
@@ -4232,7 +4232,7 @@
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>52 inch ceiling fan with light and remote downrod</t>
+          <t>52 inch ceiling fan with light and remote flush</t>
         </is>
       </c>
       <c r="B136" s="2" t="n">
@@ -4240,15 +4240,15 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>$95.93</t>
+          <t>$98.67</t>
         </is>
       </c>
       <c r="D136" s="2" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>42.4%</t>
+          <t>63.6%</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
@@ -4260,23 +4260,23 @@
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>52 inch ceiling fan with light and remote flush</t>
+          <t>52 inch ceiling fan no light</t>
         </is>
       </c>
       <c r="B137" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>$98.67</t>
+          <t>$107.57</t>
         </is>
       </c>
       <c r="D137" s="2" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>63.6%</t>
+          <t>40.6%</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
@@ -4288,23 +4288,23 @@
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>52 inch ceiling fan no light</t>
+          <t>52 inch tv console cabinet</t>
         </is>
       </c>
       <c r="B138" s="2" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>$107.57</t>
+          <t>$133.41</t>
         </is>
       </c>
       <c r="D138" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>40.6%</t>
+          <t>48.3%</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
@@ -4316,23 +4316,23 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>52 inch tv console cabinet</t>
+          <t>52 inch ceiling fan with light and remote control</t>
         </is>
       </c>
       <c r="B139" s="2" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>$133.41</t>
+          <t>$84.10</t>
         </is>
       </c>
       <c r="D139" s="2" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>48.3%</t>
+          <t>60.6%</t>
         </is>
       </c>
       <c r="F139" s="2" t="inlineStr">
@@ -4344,23 +4344,23 @@
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>52 inch ceiling fan with light and remote control</t>
+          <t>52 inch ceiling fan with led light remote control</t>
         </is>
       </c>
       <c r="B140" s="2" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>$84.10</t>
+          <t>$78.02</t>
         </is>
       </c>
       <c r="D140" s="2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>60.6%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr">
@@ -4372,7 +4372,7 @@
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>52 inch ceiling fan with led light remote control</t>
+          <t>52 inch ceiling fan with light and remote</t>
         </is>
       </c>
       <c r="B141" s="2" t="n">
@@ -4380,15 +4380,15 @@
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>$78.02</t>
+          <t>$89.41</t>
         </is>
       </c>
       <c r="D141" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>79.2%</t>
         </is>
       </c>
       <c r="F141" s="2" t="inlineStr">
@@ -4400,23 +4400,23 @@
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>52 inch ceiling fan with light and remote</t>
+          <t>control pickleball paddles</t>
         </is>
       </c>
       <c r="B142" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>$89.41</t>
+          <t>$83.11</t>
         </is>
       </c>
       <c r="D142" s="2" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>79.2%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
@@ -4428,23 +4428,23 @@
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>control pickleball paddles</t>
+          <t>portable pickleball net with wheels</t>
         </is>
       </c>
       <c r="B143" s="2" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>$83.11</t>
+          <t>$132.37</t>
         </is>
       </c>
       <c r="D143" s="2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>45.2%</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
@@ -4456,23 +4456,23 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>electronics tablets apple</t>
+          <t>wildbird baby carrier plaid</t>
         </is>
       </c>
       <c r="B144" s="2" t="n">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>$129.19</t>
+          <t>$74.95</t>
         </is>
       </c>
       <c r="D144" s="2" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>71.4%</t>
+          <t>62.5%</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
@@ -4484,23 +4484,23 @@
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>portable pickleball net with wheels</t>
+          <t>slk pickleball paddles</t>
         </is>
       </c>
       <c r="B145" s="2" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>$132.37</t>
+          <t>$89.03</t>
         </is>
       </c>
       <c r="D145" s="2" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>45.2%</t>
+          <t>54.5%</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
@@ -4512,23 +4512,23 @@
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>electronics tablets ipad apple</t>
+          <t>minoxidil foam for women</t>
         </is>
       </c>
       <c r="B146" s="2" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>$142.12</t>
+          <t>$26.97</t>
         </is>
       </c>
       <c r="D146" s="2" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>53.1%</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
@@ -4540,23 +4540,23 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>ivermectin tablets for person made in usa</t>
+          <t>joola pickleball paddle set</t>
         </is>
       </c>
       <c r="B147" s="2" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>$56.13</t>
+          <t>$103.35</t>
         </is>
       </c>
       <c r="D147" s="2" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>45.8%</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr">
@@ -4568,23 +4568,23 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>wildbird baby carrier plaid</t>
+          <t>rogaine 5% minoxidil foam</t>
         </is>
       </c>
       <c r="B148" s="2" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>$74.95</t>
+          <t>$30.07</t>
         </is>
       </c>
       <c r="D148" s="2" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>62.5%</t>
+          <t>58.6%</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr">
@@ -4596,23 +4596,23 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>slk pickleball paddles</t>
+          <t>bonide systemic granules for plants</t>
         </is>
       </c>
       <c r="B149" s="2" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>$89.03</t>
+          <t>$20.88</t>
         </is>
       </c>
       <c r="D149" s="2" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>54.5%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F149" s="2" t="inlineStr">
@@ -4624,23 +4624,23 @@
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>electronics tablets lenovo</t>
+          <t>pickleball set with net</t>
         </is>
       </c>
       <c r="B150" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>$82.56</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="C150" s="2" t="inlineStr">
-        <is>
-          <t>$212.23</t>
-        </is>
-      </c>
-      <c r="D150" s="2" t="n">
-        <v>9</v>
-      </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>52.9%</t>
+          <t>48.6%</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
@@ -4652,23 +4652,23 @@
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>minoxidil foam for women</t>
+          <t>minoxidil foam for men</t>
         </is>
       </c>
       <c r="B151" s="2" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>$26.97</t>
+          <t>$28.66</t>
         </is>
       </c>
       <c r="D151" s="2" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>53.1%</t>
+          <t>48.0%</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
@@ -4680,23 +4680,23 @@
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>joola pickleball paddle set</t>
+          <t>pickleball net portable outdoor</t>
         </is>
       </c>
       <c r="B152" s="2" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>$103.35</t>
+          <t>$88.38</t>
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>45.8%</t>
+          <t>60.6%</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
@@ -4708,23 +4708,23 @@
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>rogaine 5% minoxidil foam</t>
+          <t>pickleball net outdoor</t>
         </is>
       </c>
       <c r="B153" s="2" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>$30.07</t>
+          <t>$115.31</t>
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>58.6%</t>
+          <t>51.4%</t>
         </is>
       </c>
       <c r="F153" s="2" t="inlineStr">
@@ -4736,19 +4736,19 @@
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>bonide systemic granules for plants</t>
+          <t>garlic granules 365</t>
         </is>
       </c>
       <c r="B154" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>$20.88</t>
+          <t>$17.41</t>
         </is>
       </c>
       <c r="D154" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
@@ -4764,23 +4764,23 @@
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>ivermectin tablets for person stromectol</t>
+          <t>mjjc foam cannon</t>
         </is>
       </c>
       <c r="B155" s="2" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>$37.98</t>
+          <t>$56.16</t>
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>45.5%</t>
         </is>
       </c>
       <c r="F155" s="2" t="inlineStr">
@@ -4792,23 +4792,23 @@
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>android tablets on sale</t>
+          <t>baby monitor for car usb c</t>
         </is>
       </c>
       <c r="B156" s="2" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>$113.83</t>
+          <t>$65.73</t>
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>77.8%</t>
+          <t>46.7%</t>
         </is>
       </c>
       <c r="F156" s="2" t="inlineStr">
@@ -4820,23 +4820,23 @@
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>tablets 10 inch apple</t>
+          <t>minoxidil foam rogaine</t>
         </is>
       </c>
       <c r="B157" s="2" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>$135.19</t>
+          <t>$30.50</t>
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>73.3%</t>
+          <t>57.1%</t>
         </is>
       </c>
       <c r="F157" s="2" t="inlineStr">
@@ -4848,23 +4848,23 @@
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>pickleball set with net</t>
+          <t>minoxidil foam</t>
         </is>
       </c>
       <c r="B158" s="2" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>$82.56</t>
+          <t>$25.22</t>
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>48.6%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
@@ -4876,23 +4876,23 @@
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>minoxidil foam for men</t>
+          <t>peelers gummy candy easter</t>
         </is>
       </c>
       <c r="B159" s="2" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>$28.66</t>
+          <t>$20.46</t>
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>48.0%</t>
+          <t>66.7%</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
@@ -4904,23 +4904,23 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>pickleball net portable outdoor</t>
+          <t>minoxidil foam for women hair growth</t>
         </is>
       </c>
       <c r="B160" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>$88.38</t>
+          <t>$27.82</t>
         </is>
       </c>
       <c r="D160" s="2" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>60.6%</t>
+          <t>53.1%</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr">
@@ -4932,23 +4932,23 @@
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>ivermectin tablets for person 12 mg</t>
+          <t>portable pickleball net</t>
         </is>
       </c>
       <c r="B161" s="2" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>$87.23</t>
+          <t>$118.01</t>
         </is>
       </c>
       <c r="D161" s="2" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>59.4%</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr">
@@ -4960,23 +4960,23 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>pickleball net outdoor</t>
+          <t>scotts turf builder rapid grass tall fescue mix - combination grass seed and fertilizer for lawns, lawn seed that grows in just weeks, 5.6 lbs.</t>
         </is>
       </c>
       <c r="B162" s="2" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>$115.31</t>
+          <t>$35.49</t>
         </is>
       </c>
       <c r="D162" s="2" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>51.4%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
@@ -4988,23 +4988,23 @@
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>tablets 10 + inch apple</t>
+          <t>pickleball net set</t>
         </is>
       </c>
       <c r="B163" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>$83.02</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="C163" s="2" t="inlineStr">
-        <is>
-          <t>$74.75</t>
-        </is>
-      </c>
-      <c r="D163" s="2" t="n">
-        <v>11</v>
-      </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>68.8%</t>
+          <t>45.7%</t>
         </is>
       </c>
       <c r="F163" s="2" t="inlineStr">
@@ -5016,23 +5016,23 @@
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>garlic granules 365</t>
+          <t>minoxidil foam kirkland</t>
         </is>
       </c>
       <c r="B164" s="2" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>$17.41</t>
+          <t>$29.20</t>
         </is>
       </c>
       <c r="D164" s="2" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>48.0%</t>
         </is>
       </c>
       <c r="F164" s="2" t="inlineStr">
@@ -5044,23 +5044,23 @@
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>apple tablets on sale clearance 2025</t>
+          <t>minoxidil foam 5%</t>
         </is>
       </c>
       <c r="B165" s="2" t="n">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>$176.76</t>
+          <t>$27.11</t>
         </is>
       </c>
       <c r="D165" s="2" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
-          <t>53.8%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F165" s="2" t="inlineStr">
@@ -5072,23 +5072,23 @@
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>mjjc foam cannon</t>
+          <t>driveway pickleball set with net</t>
         </is>
       </c>
       <c r="B166" s="2" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>$56.16</t>
+          <t>$89.59</t>
         </is>
       </c>
       <c r="D166" s="2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>42.4%</t>
         </is>
       </c>
       <c r="F166" s="2" t="inlineStr">
@@ -5100,614 +5100,26 @@
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>baby monitor for car usb c</t>
+          <t>oeko-tex standard 100learn more about oeko-tex standard 100</t>
         </is>
       </c>
       <c r="B167" s="2" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>$65.73</t>
+          <t>$48.49</t>
         </is>
       </c>
       <c r="D167" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E167" s="2" t="inlineStr">
         <is>
-          <t>46.7%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F167" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" s="2" t="inlineStr">
-        <is>
-          <t>minoxidil foam rogaine</t>
-        </is>
-      </c>
-      <c r="B168" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="C168" s="2" t="inlineStr">
-        <is>
-          <t>$30.50</t>
-        </is>
-      </c>
-      <c r="D168" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="E168" s="2" t="inlineStr">
-        <is>
-          <t>57.1%</t>
-        </is>
-      </c>
-      <c r="F168" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" s="2" t="inlineStr">
-        <is>
-          <t>minoxidil foam</t>
-        </is>
-      </c>
-      <c r="B169" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="C169" s="2" t="inlineStr">
-        <is>
-          <t>$25.22</t>
-        </is>
-      </c>
-      <c r="D169" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="E169" s="2" t="inlineStr">
-        <is>
-          <t>40.0%</t>
-        </is>
-      </c>
-      <c r="F169" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" s="2" t="inlineStr">
-        <is>
-          <t>electronics tablets huawei</t>
-        </is>
-      </c>
-      <c r="B170" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="C170" s="2" t="inlineStr">
-        <is>
-          <t>$101.41</t>
-        </is>
-      </c>
-      <c r="D170" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="E170" s="2" t="inlineStr">
-        <is>
-          <t>50.0%</t>
-        </is>
-      </c>
-      <c r="F170" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" s="2" t="inlineStr">
-        <is>
-          <t>samsung tablets 10 + inch</t>
-        </is>
-      </c>
-      <c r="B171" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="C171" s="2" t="inlineStr">
-        <is>
-          <t>$201.34</t>
-        </is>
-      </c>
-      <c r="D171" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E171" s="2" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="F171" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" s="2" t="inlineStr">
-        <is>
-          <t>tablets on sale clearance 2025</t>
-        </is>
-      </c>
-      <c r="B172" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="C172" s="2" t="inlineStr">
-        <is>
-          <t>$131.75</t>
-        </is>
-      </c>
-      <c r="D172" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="E172" s="2" t="inlineStr">
-        <is>
-          <t>72.2%</t>
-        </is>
-      </c>
-      <c r="F172" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" s="2" t="inlineStr">
-        <is>
-          <t>tablets for kids 10 + inch</t>
-        </is>
-      </c>
-      <c r="B173" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="C173" s="2" t="inlineStr">
-        <is>
-          <t>$76.14</t>
-        </is>
-      </c>
-      <c r="D173" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="E173" s="2" t="inlineStr">
-        <is>
-          <t>57.9%</t>
-        </is>
-      </c>
-      <c r="F173" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" s="2" t="inlineStr">
-        <is>
-          <t>peelers gummy candy easter</t>
-        </is>
-      </c>
-      <c r="B174" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="C174" s="2" t="inlineStr">
-        <is>
-          <t>$20.46</t>
-        </is>
-      </c>
-      <c r="D174" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E174" s="2" t="inlineStr">
-        <is>
-          <t>66.7%</t>
-        </is>
-      </c>
-      <c r="F174" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" s="2" t="inlineStr">
-        <is>
-          <t>minoxidil foam for women hair growth</t>
-        </is>
-      </c>
-      <c r="B175" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="C175" s="2" t="inlineStr">
-        <is>
-          <t>$27.82</t>
-        </is>
-      </c>
-      <c r="D175" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="E175" s="2" t="inlineStr">
-        <is>
-          <t>53.1%</t>
-        </is>
-      </c>
-      <c r="F175" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="2" t="inlineStr">
-        <is>
-          <t>portable pickleball net</t>
-        </is>
-      </c>
-      <c r="B176" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="C176" s="2" t="inlineStr">
-        <is>
-          <t>$118.01</t>
-        </is>
-      </c>
-      <c r="D176" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="E176" s="2" t="inlineStr">
-        <is>
-          <t>59.4%</t>
-        </is>
-      </c>
-      <c r="F176" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" s="2" t="inlineStr">
-        <is>
-          <t>scotts turf builder rapid grass tall fescue mix - combination grass seed and fertilizer for lawns, lawn seed that grows in just weeks, 5.6 lbs.</t>
-        </is>
-      </c>
-      <c r="B177" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C177" s="2" t="inlineStr">
-        <is>
-          <t>$35.49</t>
-        </is>
-      </c>
-      <c r="D177" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E177" s="2" t="inlineStr">
-        <is>
-          <t>50.0%</t>
-        </is>
-      </c>
-      <c r="F177" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="2" t="inlineStr">
-        <is>
-          <t>pickleball net set</t>
-        </is>
-      </c>
-      <c r="B178" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="C178" s="2" t="inlineStr">
-        <is>
-          <t>$83.02</t>
-        </is>
-      </c>
-      <c r="D178" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="E178" s="2" t="inlineStr">
-        <is>
-          <t>45.7%</t>
-        </is>
-      </c>
-      <c r="F178" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="2" t="inlineStr">
-        <is>
-          <t>ivermectin tablets for person 12 mg 100</t>
-        </is>
-      </c>
-      <c r="B179" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C179" s="2" t="inlineStr">
-        <is>
-          <t>$75.53</t>
-        </is>
-      </c>
-      <c r="D179" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E179" s="2" t="inlineStr">
-        <is>
-          <t>40.0%</t>
-        </is>
-      </c>
-      <c r="F179" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" s="2" t="inlineStr">
-        <is>
-          <t>kindle tablets 10 inch fire hd new</t>
-        </is>
-      </c>
-      <c r="B180" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="C180" s="2" t="inlineStr">
-        <is>
-          <t>$77.68</t>
-        </is>
-      </c>
-      <c r="D180" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="E180" s="2" t="inlineStr">
-        <is>
-          <t>63.6%</t>
-        </is>
-      </c>
-      <c r="F180" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" s="2" t="inlineStr">
-        <is>
-          <t>samsung tablets 10 inch</t>
-        </is>
-      </c>
-      <c r="B181" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="C181" s="2" t="inlineStr">
-        <is>
-          <t>$166.25</t>
-        </is>
-      </c>
-      <c r="D181" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="E181" s="2" t="inlineStr">
-        <is>
-          <t>88.2%</t>
-        </is>
-      </c>
-      <c r="F181" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" s="2" t="inlineStr">
-        <is>
-          <t>ivermectin tablets for person otc</t>
-        </is>
-      </c>
-      <c r="B182" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="C182" s="2" t="inlineStr">
-        <is>
-          <t>$52.84</t>
-        </is>
-      </c>
-      <c r="D182" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E182" s="2" t="inlineStr">
-        <is>
-          <t>45.5%</t>
-        </is>
-      </c>
-      <c r="F182" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" s="2" t="inlineStr">
-        <is>
-          <t>minoxidil foam kirkland</t>
-        </is>
-      </c>
-      <c r="B183" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="C183" s="2" t="inlineStr">
-        <is>
-          <t>$29.20</t>
-        </is>
-      </c>
-      <c r="D183" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E183" s="2" t="inlineStr">
-        <is>
-          <t>48.0%</t>
-        </is>
-      </c>
-      <c r="F183" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" s="2" t="inlineStr">
-        <is>
-          <t>minoxidil foam 5%</t>
-        </is>
-      </c>
-      <c r="B184" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="C184" s="2" t="inlineStr">
-        <is>
-          <t>$27.11</t>
-        </is>
-      </c>
-      <c r="D184" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E184" s="2" t="inlineStr">
-        <is>
-          <t>40.0%</t>
-        </is>
-      </c>
-      <c r="F184" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" s="2" t="inlineStr">
-        <is>
-          <t>driveway pickleball set with net</t>
-        </is>
-      </c>
-      <c r="B185" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="C185" s="2" t="inlineStr">
-        <is>
-          <t>$89.59</t>
-        </is>
-      </c>
-      <c r="D185" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="E185" s="2" t="inlineStr">
-        <is>
-          <t>42.4%</t>
-        </is>
-      </c>
-      <c r="F185" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" s="2" t="inlineStr">
-        <is>
-          <t>oeko-tex standard 100learn more about oeko-tex standard 100</t>
-        </is>
-      </c>
-      <c r="B186" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C186" s="2" t="inlineStr">
-        <is>
-          <t>$48.49</t>
-        </is>
-      </c>
-      <c r="D186" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E186" s="2" t="inlineStr">
-        <is>
-          <t>50.0%</t>
-        </is>
-      </c>
-      <c r="F186" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" s="2" t="inlineStr">
-        <is>
-          <t>tablets 10 + inch for kids</t>
-        </is>
-      </c>
-      <c r="B187" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="C187" s="2" t="inlineStr">
-        <is>
-          <t>$78.72</t>
-        </is>
-      </c>
-      <c r="D187" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="E187" s="2" t="inlineStr">
-        <is>
-          <t>57.9%</t>
-        </is>
-      </c>
-      <c r="F187" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" s="2" t="inlineStr">
-        <is>
-          <t>ivermectin tablets for person without prescription</t>
-        </is>
-      </c>
-      <c r="B188" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C188" s="2" t="inlineStr">
-        <is>
-          <t>$52.89</t>
-        </is>
-      </c>
-      <c r="D188" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E188" s="2" t="inlineStr">
-        <is>
-          <t>66.7%</t>
-        </is>
-      </c>
-      <c r="F188" s="2" t="inlineStr">
         <is>
           <t>✅ GİRİLEBİLİR</t>
         </is>

</xml_diff>

<commit_message>
minoxidil samsung 3days silindi
</commit_message>
<xml_diff>
--- a/output/amazon_niche_rapor_2026-03-31.xlsx
+++ b/output/amazon_niche_rapor_2026-03-31.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F167"/>
+  <dimension ref="A1:F144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -536,23 +536,23 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>rozino 3 day nail care with gel overlay</t>
+          <t>baby monitor for car seats with usb connectivity</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>$12.94</t>
+          <t>$78.01</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>41.7%</t>
+          <t>60.0%</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -564,23 +564,23 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>baby monitor for car seats with usb connectivity</t>
+          <t>in wall cable management kit surge protector</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>$78.01</t>
+          <t>$47.37</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>45.5%</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -592,23 +592,23 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>in wall cable management kit surge protector</t>
+          <t>baby monitor for carplay</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>$47.37</t>
+          <t>$100.64</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>68.4%</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -620,23 +620,23 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>baby monitor for carplay</t>
+          <t>cat bed desk mount</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>$100.64</t>
+          <t>$38.41</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>68.4%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -648,7 +648,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>cat bed desk mount</t>
+          <t>cat bed for desk attachment</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -656,15 +656,15 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>$38.41</t>
+          <t>$36.05</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>45.8%</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -676,7 +676,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>cat bed for desk attachment</t>
+          <t>cat wall mounted shelves and perches</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
@@ -684,15 +684,15 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>$36.05</t>
+          <t>$63.08</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>45.8%</t>
+          <t>41.7%</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -704,7 +704,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>cat wall mounted shelves and perches</t>
+          <t>facial roller massager with red light</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -712,15 +712,15 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>$63.08</t>
+          <t>$46.09</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>41.7%</t>
+          <t>54.2%</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -732,7 +732,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>facial roller massager with red light</t>
+          <t>exercise equipment for women kit</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
@@ -740,15 +740,15 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>$46.09</t>
+          <t>$32.54</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>54.2%</t>
+          <t>41.7%</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -760,23 +760,23 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>exercise equipment for women kit</t>
+          <t>100 count prefilled easter eggs chocolate</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>$32.54</t>
+          <t>$35.35</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>41.7%</t>
+          <t>60.6%</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -788,23 +788,23 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>100 count prefilled easter eggs chocolate</t>
+          <t>battery powered cordless lawn mowers small</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>$35.35</t>
+          <t>$155.67</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>60.6%</t>
+          <t>44.4%</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -816,23 +816,23 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>battery powered cordless lawn mowers small</t>
+          <t>bird feeders for outdoors with camera</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>$155.67</t>
+          <t>$75.72</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>44.4%</t>
+          <t>47.6%</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -844,23 +844,23 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>bird feeders for outdoors with camera</t>
+          <t>battery powered sprayer backpack</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>$75.72</t>
+          <t>$106.06</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>47.6%</t>
+          <t>66.7%</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -872,7 +872,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>battery powered sprayer backpack</t>
+          <t>rootling baby feeding pillow</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -880,15 +880,15 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>$106.06</t>
+          <t>$41.02</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>41.7%</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -900,23 +900,23 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>rootling baby feeding pillow</t>
+          <t>exercise equipment for seniors sitting</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>$41.02</t>
+          <t>$85.41</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>41.7%</t>
+          <t>53.3%</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -928,23 +928,23 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>rozino keratin 3 day nail care gloss peachcroft</t>
+          <t>fsa or hsa eligible items only household</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>$13.73</t>
+          <t>$110.98</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>45.8%</t>
+          <t>46.9%</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -956,23 +956,23 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>exercise equipment for seniors sitting</t>
+          <t>indoor, outdoor wireless dog fence</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>$85.41</t>
+          <t>$158.35</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>53.3%</t>
+          <t>48.0%</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -984,23 +984,23 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>fsa or hsa eligible items only household</t>
+          <t>bird feeder with camera solar powered</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>$110.98</t>
+          <t>$90.03</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>46.9%</t>
+          <t>46.7%</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1012,23 +1012,23 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>rozino keratin 3 day nail care polish</t>
+          <t>battery powered lawn mower cordless</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>$13.69</t>
+          <t>$165.16</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1040,23 +1040,23 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>indoor, outdoor wireless dog fence</t>
+          <t>smart bird feeder with camera solar powered</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>$158.35</t>
+          <t>$76.66</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>48.0%</t>
+          <t>52.4%</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1068,23 +1068,23 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>rozino keratin 3 day nail care gloss</t>
+          <t>baby feeding pillow reflux</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>$12.88</t>
+          <t>$49.66</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>45.8%</t>
+          <t>51.5%</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1096,23 +1096,23 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>rozino 3 day nail care keratin</t>
+          <t>nanit baby monitor wall mount</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>$14.01</t>
+          <t>$118.27</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>40.6%</t>
+          <t>46.7%</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1124,23 +1124,23 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>bird feeder with camera solar powered</t>
+          <t>100 count prefilled easter eggs</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>$90.03</t>
+          <t>$30.09</t>
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>46.7%</t>
+          <t>62.1%</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1152,19 +1152,19 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>battery powered lawn mower cordless</t>
+          <t>wooden chopping boards like books</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>$165.16</t>
+          <t>$67.94</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
@@ -1180,23 +1180,23 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>smart bird feeder with camera solar powered</t>
+          <t>plant stand with grow lights for indoor growing</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>$76.66</t>
+          <t>$63.28</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>52.4%</t>
+          <t>57.6%</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1208,7 +1208,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>baby feeding pillow reflux</t>
+          <t>sourdough bread baking supplies dutch oven</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>$49.66</t>
+          <t>$54.63</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
@@ -1236,23 +1236,23 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>nanit baby monitor wall mount</t>
+          <t>cat bed for desktop</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>$118.27</t>
+          <t>$34.57</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>46.7%</t>
+          <t>42.3%</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1264,23 +1264,23 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>100 count prefilled easter eggs</t>
+          <t>battery powered lawn mower 80v</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>$30.09</t>
+          <t>$139.66</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>62.1%</t>
+          <t>66.7%</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1292,23 +1292,23 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>wooden chopping boards like books</t>
+          <t>cat bed desk mount large</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>$67.94</t>
+          <t>$37.88</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>45.5%</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1320,7 +1320,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>plant stand with grow lights for indoor growing</t>
+          <t>tall plant stand with grow light</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1328,15 +1328,15 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>$63.28</t>
+          <t>$66.93</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>57.6%</t>
+          <t>42.4%</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1348,23 +1348,23 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>sourdough bread baking supplies dutch oven</t>
+          <t>smart bird feeder with camera</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>$54.63</t>
+          <t>$95.33</t>
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>51.5%</t>
+          <t>46.7%</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1376,23 +1376,23 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>cat bed for desktop</t>
+          <t>cat bed for desk with clamp</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>$34.57</t>
+          <t>$37.31</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>42.3%</t>
+          <t>45.5%</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1404,23 +1404,23 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>battery powered lawn mower 80v</t>
+          <t>wireless baby monitor for car with night vision</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>$139.66</t>
+          <t>$78.30</t>
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>59.1%</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -1432,7 +1432,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>cat bed desk mount large</t>
+          <t>plant stand indoor with grow lights black</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>$37.88</t>
+          <t>$61.54</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
@@ -1460,23 +1460,23 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>3 days nail care - keratin amino acid formula rozino</t>
+          <t>bird buddy smart bird feeder with camera</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>$13.71</t>
+          <t>$108.96</t>
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>48.5%</t>
+          <t>48.4%</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -1488,23 +1488,23 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>tall plant stand with grow light</t>
+          <t>100 count easter eggs filled</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>$66.93</t>
+          <t>$30.92</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>42.4%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -1516,23 +1516,23 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>rozino keratin 3 day nail care fungus</t>
+          <t>100 count prefilled easter eggs candy</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>$13.97</t>
+          <t>$38.95</t>
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>43.5%</t>
+          <t>62.5%</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1544,23 +1544,23 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>rozino keratin 3 day nail care</t>
+          <t>battery powered lawn mower 21 inch</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>$12.48</t>
+          <t>$144.59</t>
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>40.6%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -1572,23 +1572,23 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>smart bird feeder with camera</t>
+          <t>100 count easter eggs prefilled with candy</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>$95.33</t>
+          <t>$35.14</t>
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>46.7%</t>
+          <t>57.6%</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -1600,23 +1600,23 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>cat bed for desk with clamp</t>
+          <t>baby monitor for car carplay</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>$37.31</t>
+          <t>$99.79</t>
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>60.0%</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -1628,23 +1628,23 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>wireless baby monitor for car with night vision</t>
+          <t>plant stand indoor with grow lights</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>$78.30</t>
+          <t>$55.68</t>
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>59.1%</t>
+          <t>62.5%</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -1656,23 +1656,23 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>plant stand indoor with grow lights black</t>
+          <t>mabe baby carrier mocha</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>$61.54</t>
+          <t>$71.15</t>
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>70.8%</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -1684,23 +1684,23 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>bird buddy smart bird feeder with camera</t>
+          <t>jarritos zero sugar</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>31</v>
+        <v>2</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>$108.96</t>
+          <t>$28.99</t>
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>48.4%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -1712,23 +1712,23 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>100 count easter eggs filled</t>
+          <t>in wall cable management kit with power</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>$30.92</t>
+          <t>$46.59</t>
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>46.7%</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -1740,23 +1740,23 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>100 count prefilled easter eggs candy</t>
+          <t>battery powered sprayer 2 gallon</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>$38.95</t>
+          <t>$43.10</t>
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>62.5%</t>
+          <t>41.9%</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -1768,23 +1768,23 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>battery powered lawn mower 21 inch</t>
+          <t>titanium cutting boards for kitchen</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>$144.59</t>
+          <t>$47.57</t>
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>42.4%</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -1796,23 +1796,23 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>100 count easter eggs prefilled with candy</t>
+          <t>baby monitor for car play</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>$35.14</t>
+          <t>$94.56</t>
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>57.6%</t>
+          <t>64.3%</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -1824,23 +1824,23 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>baby monitor for car carplay</t>
+          <t>taima titanium cutting board</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>$99.79</t>
+          <t>$58.68</t>
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>57.6%</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -1852,23 +1852,23 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>plant stand indoor with grow lights</t>
+          <t>lazy boy outdoor furniture cushions</t>
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>$55.68</t>
+          <t>$69.55</t>
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>62.5%</t>
+          <t>46.4%</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -1880,7 +1880,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>mabe baby carrier mocha</t>
+          <t>hosereel retractable garden hose</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -1888,15 +1888,15 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>$71.15</t>
+          <t>$104.14</t>
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>70.8%</t>
+          <t>66.7%</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -1908,23 +1908,23 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>jarritos zero sugar</t>
+          <t>baby feeding pillow anti overflow</t>
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>$28.99</t>
+          <t>$39.12</t>
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>40.6%</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -1936,23 +1936,23 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>in wall cable management kit with power</t>
+          <t>cat bed for desk attachment purple</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>$46.59</t>
+          <t>$37.13</t>
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>46.7%</t>
+          <t>53.3%</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -1964,23 +1964,23 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>battery powered sprayer 2 gallon</t>
+          <t>3 sizes of metal arch backdrop stand</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>$43.10</t>
+          <t>$46.22</t>
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>41.9%</t>
+          <t>57.1%</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -1992,23 +1992,23 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>titanium cutting boards for kitchen</t>
+          <t>sports garage organizer white wheels backpack hook</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>$47.57</t>
+          <t>$69.49</t>
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>42.4%</t>
+          <t>52.9%</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -2020,23 +2020,23 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>rozino keratin 3 day nail care set</t>
+          <t>adjustable dumbbell rack</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>$14.97</t>
+          <t>$84.46</t>
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>44.8%</t>
+          <t>42.4%</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -2048,23 +2048,23 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>baby monitor for car play</t>
+          <t>bird feeder with camera</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>$94.56</t>
+          <t>$78.64</t>
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>64.3%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -2076,23 +2076,23 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>taima titanium cutting board</t>
+          <t>humming bird feeder with camera</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>$58.68</t>
+          <t>$103.17</t>
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>57.6%</t>
+          <t>46.9%</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -2104,23 +2104,23 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>lazy boy outdoor furniture cushions</t>
+          <t>bird feeder with camera no subscription</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>$69.55</t>
+          <t>$73.04</t>
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>46.4%</t>
+          <t>52.4%</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -2132,23 +2132,23 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>hosereel retractable garden hose</t>
+          <t>book cutting board set</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>$104.14</t>
+          <t>$73.71</t>
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>45.5%</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -2160,23 +2160,23 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>baby feeding pillow anti overflow</t>
+          <t>cellulite massage tool electric</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>$39.12</t>
+          <t>$39.45</t>
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>40.6%</t>
+          <t>45.8%</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -2188,23 +2188,23 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>cat bed for desk attachment purple</t>
+          <t>lighted plant stand indoor</t>
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>$37.13</t>
+          <t>$134.79</t>
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>53.3%</t>
+          <t>46.4%</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -2216,19 +2216,19 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>3 sizes of metal arch backdrop stand</t>
+          <t>perineal massage tool kiwi</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>$46.22</t>
+          <t>$37.85</t>
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
@@ -2244,23 +2244,23 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>rozino keratin 3 day nail care carb nail gloss</t>
+          <t>forestry practices buffet cabinet</t>
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>$13.42</t>
+          <t>$104.29</t>
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>45.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -2272,23 +2272,23 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>sports garage organizer white wheels backpack hook</t>
+          <t>100 count pre filled easter eggs candy</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>$69.49</t>
+          <t>$29.35</t>
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>52.9%</t>
+          <t>55.9%</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -2300,23 +2300,23 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>3 days nail care oil</t>
+          <t>sponsored camara</t>
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>$12.90</t>
+          <t>$99.85</t>
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>46.7%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -2328,23 +2328,23 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>3 days nail care oil with keratin</t>
+          <t>baby monitor for car seat</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>$12.90</t>
+          <t>$68.17</t>
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>46.7%</t>
+          <t>59.1%</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -2356,23 +2356,23 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>adjustable dumbbell rack</t>
+          <t>battery powered sprayer 4 gallon</t>
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>$84.46</t>
+          <t>$98.33</t>
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>42.4%</t>
+          <t>62.5%</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -2384,23 +2384,23 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>bird feeder with camera</t>
+          <t>cat bed desk mount folding</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>$78.64</t>
+          <t>$37.05</t>
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>45.2%</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -2412,23 +2412,23 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>humming bird feeder with camera</t>
+          <t>small battery powered lawn mower</t>
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>$103.17</t>
+          <t>$153.69</t>
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>46.9%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -2440,23 +2440,23 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>bird feeder with camera no subscription</t>
+          <t>skincare device fsa</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>$73.04</t>
+          <t>$129.79</t>
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>52.4%</t>
+          <t>68.4%</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -2468,7 +2468,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>book cutting board set</t>
+          <t>humming bird feeders for outdoors with camera</t>
         </is>
       </c>
       <c r="B73" s="2" t="n">
@@ -2476,15 +2476,15 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>$73.71</t>
+          <t>$93.71</t>
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>63.6%</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -2496,15 +2496,15 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>cellulite massage tool electric</t>
+          <t>cat bed desk mounted</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>$39.45</t>
+          <t>$37.46</t>
         </is>
       </c>
       <c r="D74" s="2" t="n">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>45.8%</t>
+          <t>47.8%</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -2524,23 +2524,23 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>lighted plant stand indoor</t>
+          <t>cellulite massage tool suction cup</t>
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>$134.79</t>
+          <t>$34.88</t>
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>46.4%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -2552,23 +2552,23 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>3 days nail care - keratin amino acid formula</t>
+          <t>baby monitor for car 2 cameras</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>$13.07</t>
+          <t>$62.69</t>
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>56.7%</t>
+          <t>72.7%</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -2580,23 +2580,23 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>perineal massage tool kiwi</t>
+          <t>retractable garden hose 5/8</t>
         </is>
       </c>
       <c r="B77" s="2" t="n">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>$37.85</t>
+          <t>$132.59</t>
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>57.1%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -2608,23 +2608,23 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>forestry practices buffet cabinet</t>
+          <t>mugwort seeds</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>$104.29</t>
+          <t>$47.49</t>
         </is>
       </c>
       <c r="D78" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -2636,23 +2636,23 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>100 count pre filled easter eggs candy</t>
+          <t>100 count prefilled easter eggs with toys</t>
         </is>
       </c>
       <c r="B79" s="2" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>$29.35</t>
+          <t>$32.14</t>
         </is>
       </c>
       <c r="D79" s="2" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>55.9%</t>
+          <t>57.7%</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -2664,23 +2664,23 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>sponsored camara</t>
+          <t>cat bed desk mount heavy duty</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>$99.85</t>
+          <t>$39.17</t>
         </is>
       </c>
       <c r="D80" s="2" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>43.8%</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -2692,23 +2692,23 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>baby monitor for car seat</t>
+          <t>83 inch oled tv g series</t>
         </is>
       </c>
       <c r="B81" s="2" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>$68.17</t>
+          <t>$159.43</t>
         </is>
       </c>
       <c r="D81" s="2" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>59.1%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -2720,23 +2720,23 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>battery powered sprayer 4 gallon</t>
+          <t>removedor de verrugas genitales vph</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>$98.33</t>
+          <t>$24.32</t>
         </is>
       </c>
       <c r="D82" s="2" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>62.5%</t>
+          <t>66.7%</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -2748,23 +2748,23 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>cat bed desk mount folding</t>
+          <t>renogy solar panels</t>
         </is>
       </c>
       <c r="B83" s="2" t="n">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>$37.05</t>
+          <t>$210.82</t>
         </is>
       </c>
       <c r="D83" s="2" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>45.2%</t>
+          <t>43.8%</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -2776,23 +2776,23 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>small battery powered lawn mower</t>
+          <t>3k monitor 24 inch 3840 x 2160</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>$273.24</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>$153.69</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>70.0%</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -2804,23 +2804,23 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>skincare device fsa</t>
+          <t>zep stainless steel cleaner</t>
         </is>
       </c>
       <c r="B85" s="2" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>$129.79</t>
+          <t>$13.98</t>
         </is>
       </c>
       <c r="D85" s="2" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>68.4%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -2832,23 +2832,23 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>humming bird feeders for outdoors with camera</t>
+          <t>3k watt amp big bass</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>$93.71</t>
+          <t>$215.55</t>
         </is>
       </c>
       <c r="D86" s="2" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>63.6%</t>
+          <t>56.2%</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -2860,23 +2860,23 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>cat bed desk mounted</t>
+          <t>2026 mahjong card official american</t>
         </is>
       </c>
       <c r="B87" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>$37.46</t>
+          <t>$28.37</t>
         </is>
       </c>
       <c r="D87" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>47.8%</t>
+          <t>41.7%</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -2888,19 +2888,19 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>cellulite massage tool suction cup</t>
+          <t>3k taramps amp bass</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>$34.88</t>
+          <t>$251.81</t>
         </is>
       </c>
       <c r="D88" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
@@ -2916,23 +2916,23 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>baby monitor for car 2 cameras</t>
+          <t>3k watt amp wiring kit ofc</t>
         </is>
       </c>
       <c r="B89" s="2" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>$62.69</t>
+          <t>$79.87</t>
         </is>
       </c>
       <c r="D89" s="2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>72.7%</t>
+          <t>46.2%</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
@@ -2944,23 +2944,23 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>retractable garden hose 5/8</t>
+          <t>3k bass amp</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>$132.59</t>
+          <t>$205.96</t>
         </is>
       </c>
       <c r="D90" s="2" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -2972,23 +2972,23 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>rozino 3 day nail care keratin amino acid</t>
+          <t>83 inch oled tv g4</t>
         </is>
       </c>
       <c r="B91" s="2" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>$13.68</t>
+          <t>$39.99</t>
         </is>
       </c>
       <c r="D91" s="2" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
@@ -3000,23 +3000,23 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>mugwort seeds</t>
+          <t>83 inch oled tv gaming</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>$47.49</t>
+          <t>$172.64</t>
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -3028,23 +3028,23 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>100 count prefilled easter eggs with toys</t>
+          <t>3k monitor 240hz</t>
         </is>
       </c>
       <c r="B93" s="2" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>$32.14</t>
+          <t>$338.03</t>
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>57.7%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
@@ -3056,23 +3056,23 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>cat bed desk mount heavy duty</t>
+          <t>sprayway stainless steel cleaner</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>$39.17</t>
+          <t>$17.37</t>
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>43.8%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
@@ -3084,23 +3084,23 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>83 inch oled tv g series</t>
+          <t>66 inch tv</t>
         </is>
       </c>
       <c r="B95" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>$103.12</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C95" s="2" t="inlineStr">
-        <is>
-          <t>$159.43</t>
-        </is>
-      </c>
-      <c r="D95" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>66.7%</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -3112,23 +3112,23 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>removedor de verrugas genitales vph</t>
+          <t>xxxl stainless steel litter box</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>$24.32</t>
+          <t>$94.60</t>
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>48.0%</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
@@ -3140,23 +3140,23 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>renogy solar panels</t>
+          <t>83 inch oled tv c5</t>
         </is>
       </c>
       <c r="B97" s="2" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>$210.82</t>
+          <t>$108.96</t>
         </is>
       </c>
       <c r="D97" s="2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>43.8%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
@@ -3168,23 +3168,23 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>3k monitor 24 inch 3840 x 2160</t>
+          <t>gardening organizer cart</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>$273.24</t>
+          <t>$72.95</t>
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>47.1%</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
@@ -3196,23 +3196,23 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>zep stainless steel cleaner</t>
+          <t>plug in solar panels for homes</t>
         </is>
       </c>
       <c r="B99" s="2" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>$13.98</t>
+          <t>$143.94</t>
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>60.0%</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
@@ -3224,23 +3224,23 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>3k watt amp big bass</t>
+          <t>66 roots journey bible study</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>$215.55</t>
+          <t>$17.41</t>
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>56.2%</t>
+          <t>41.7%</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -3252,23 +3252,23 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>2026 mahjong card official american</t>
+          <t>3k amplifier 4 channel</t>
         </is>
       </c>
       <c r="B101" s="2" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>$28.37</t>
+          <t>$181.03</t>
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>41.7%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
@@ -3280,23 +3280,23 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>3k taramps amp bass</t>
+          <t>stainless steel litter box sifting</t>
         </is>
       </c>
       <c r="B102" s="2" t="n">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>$251.81</t>
+          <t>$70.33</t>
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>44.1%</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
@@ -3308,23 +3308,23 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>3k watt amp wiring kit ofc</t>
+          <t>3k taramps amp 4 channel</t>
         </is>
       </c>
       <c r="B103" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>$79.87</t>
+          <t>$200.81</t>
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>46.2%</t>
+          <t>46.7%</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -3336,23 +3336,23 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>3k bass amp</t>
+          <t>3k bass amp taramps</t>
         </is>
       </c>
       <c r="B104" s="2" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>$205.96</t>
+          <t>$251.94</t>
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
@@ -3364,23 +3364,23 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>83 inch oled tv samsung</t>
+          <t>83 oled lg</t>
         </is>
       </c>
       <c r="B105" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>$486.18</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C105" s="2" t="inlineStr">
-        <is>
-          <t>$2522.85</t>
-        </is>
-      </c>
-      <c r="D105" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
@@ -3392,19 +3392,19 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>83 inch oled tv g4</t>
+          <t>2032 battery 2 pack</t>
         </is>
       </c>
       <c r="B106" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>$39.99</t>
+          <t>$29.36</t>
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
@@ -3420,23 +3420,23 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>83 inch oled tv gaming</t>
+          <t>66 page bible study guide extra large print</t>
         </is>
       </c>
       <c r="B107" s="2" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>$172.64</t>
+          <t>$19.91</t>
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>43.5%</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
@@ -3448,23 +3448,23 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>3k monitor 240hz</t>
+          <t>kettlebell rack stand only</t>
         </is>
       </c>
       <c r="B108" s="2" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>$338.03</t>
+          <t>$63.81</t>
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>45.5%</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
@@ -3476,23 +3476,23 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>sprayway stainless steel cleaner</t>
+          <t>66 inch tv console</t>
         </is>
       </c>
       <c r="B109" s="2" t="n">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>$17.37</t>
+          <t>$118.36</t>
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>44.8%</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
@@ -3504,23 +3504,23 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>66 inch tv</t>
+          <t>katori titanium cutting board</t>
         </is>
       </c>
       <c r="B110" s="2" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>$103.12</t>
+          <t>$46.81</t>
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>45.5%</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
@@ -3532,23 +3532,23 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>xxxl stainless steel litter box</t>
+          <t>3k taramps amp 2 ohm</t>
         </is>
       </c>
       <c r="B111" s="2" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>$94.60</t>
+          <t>$222.78</t>
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>48.0%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
@@ -3560,23 +3560,23 @@
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>83 inch oled tv c5</t>
+          <t>plug in solar panels</t>
         </is>
       </c>
       <c r="B112" s="2" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>$108.96</t>
+          <t>$147.84</t>
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>63.6%</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
@@ -3588,23 +3588,23 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>gardening organizer cart</t>
+          <t>3k taramps amp 1 ohm</t>
         </is>
       </c>
       <c r="B113" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>$72.95</t>
+          <t>$195.43</t>
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>47.1%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F113" s="2" t="inlineStr">
@@ -3616,23 +3616,23 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>plug in solar panels for homes</t>
+          <t>3k taramps amp 4 ohm</t>
         </is>
       </c>
       <c r="B114" s="2" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>$143.94</t>
+          <t>$198.57</t>
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>42.1%</t>
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr">
@@ -3644,23 +3644,23 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>66 roots journey bible study</t>
+          <t>3k amp 2 channel</t>
         </is>
       </c>
       <c r="B115" s="2" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>$17.41</t>
+          <t>$189.54</t>
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>41.7%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F115" s="2" t="inlineStr">
@@ -3672,19 +3672,19 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>3k amplifier 4 channel</t>
+          <t>3k amp wiring kit</t>
         </is>
       </c>
       <c r="B116" s="2" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>$181.03</t>
+          <t>$47.04</t>
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
@@ -3700,23 +3700,23 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>stainless steel litter box sifting</t>
+          <t>83 inch oled tvs</t>
         </is>
       </c>
       <c r="B117" s="2" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>$70.33</t>
+          <t>$135.49</t>
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>44.1%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
@@ -3728,23 +3728,23 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>3k taramps amp 4 channel</t>
+          <t>4.64.6 out of 5 stars(173)300+ bought in past month</t>
         </is>
       </c>
       <c r="B118" s="2" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>$200.81</t>
+          <t>$86.99</t>
         </is>
       </c>
       <c r="D118" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>46.7%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="F118" s="2" t="inlineStr">
@@ -3756,23 +3756,23 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>3k bass amp taramps</t>
+          <t>52 inch ceiling fan with light and remote white</t>
         </is>
       </c>
       <c r="B119" s="2" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>$251.94</t>
+          <t>$94.67</t>
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>40.6%</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">
@@ -3784,23 +3784,23 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>83 oled lg</t>
+          <t>52 inch ceiling fan with light and remote downrod</t>
         </is>
       </c>
       <c r="B120" s="2" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>$486.18</t>
+          <t>$95.93</t>
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>42.4%</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
@@ -3812,23 +3812,23 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>2032 battery 2 pack</t>
+          <t>52 inch ceiling fan with light and remote flush</t>
         </is>
       </c>
       <c r="B121" s="2" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>$29.36</t>
+          <t>$98.67</t>
         </is>
       </c>
       <c r="D121" s="2" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>63.6%</t>
         </is>
       </c>
       <c r="F121" s="2" t="inlineStr">
@@ -3840,23 +3840,23 @@
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>66 page bible study guide extra large print</t>
+          <t>52 inch ceiling fan no light</t>
         </is>
       </c>
       <c r="B122" s="2" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>$19.91</t>
+          <t>$107.57</t>
         </is>
       </c>
       <c r="D122" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>43.5%</t>
+          <t>40.6%</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
@@ -3868,23 +3868,23 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>kettlebell rack stand only</t>
+          <t>52 inch tv console cabinet</t>
         </is>
       </c>
       <c r="B123" s="2" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>$63.81</t>
+          <t>$133.41</t>
         </is>
       </c>
       <c r="D123" s="2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>48.3%</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
@@ -3896,23 +3896,23 @@
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>66 inch tv console</t>
+          <t>52 inch ceiling fan with light and remote control</t>
         </is>
       </c>
       <c r="B124" s="2" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>$118.36</t>
+          <t>$84.10</t>
         </is>
       </c>
       <c r="D124" s="2" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>44.8%</t>
+          <t>60.6%</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
@@ -3924,23 +3924,23 @@
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>katori titanium cutting board</t>
+          <t>52 inch ceiling fan with led light remote control</t>
         </is>
       </c>
       <c r="B125" s="2" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>$46.81</t>
+          <t>$78.02</t>
         </is>
       </c>
       <c r="D125" s="2" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
@@ -3952,23 +3952,23 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>3k taramps amp 2 ohm</t>
+          <t>52 inch ceiling fan with light and remote</t>
         </is>
       </c>
       <c r="B126" s="2" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>$222.78</t>
+          <t>$89.41</t>
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>79.2%</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
@@ -3980,23 +3980,23 @@
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>plug in solar panels</t>
+          <t>control pickleball paddles</t>
         </is>
       </c>
       <c r="B127" s="2" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>$147.84</t>
+          <t>$83.11</t>
         </is>
       </c>
       <c r="D127" s="2" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>63.6%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
@@ -4008,23 +4008,23 @@
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>3k taramps amp 1 ohm</t>
+          <t>portable pickleball net with wheels</t>
         </is>
       </c>
       <c r="B128" s="2" t="n">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>$195.43</t>
+          <t>$132.37</t>
         </is>
       </c>
       <c r="D128" s="2" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>45.2%</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
@@ -4036,23 +4036,23 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>3k taramps amp 4 ohm</t>
+          <t>wildbird baby carrier plaid</t>
         </is>
       </c>
       <c r="B129" s="2" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>$198.57</t>
+          <t>$74.95</t>
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>42.1%</t>
+          <t>62.5%</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
@@ -4064,23 +4064,23 @@
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>3k amp 2 channel</t>
+          <t>slk pickleball paddles</t>
         </is>
       </c>
       <c r="B130" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>$189.54</t>
+          <t>$89.03</t>
         </is>
       </c>
       <c r="D130" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>54.5%</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
@@ -4092,23 +4092,23 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>3k amp wiring kit</t>
+          <t>joola pickleball paddle set</t>
         </is>
       </c>
       <c r="B131" s="2" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>$47.04</t>
+          <t>$103.35</t>
         </is>
       </c>
       <c r="D131" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>45.8%</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
@@ -4120,23 +4120,23 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>83 inch oled tvs</t>
+          <t>bonide systemic granules for plants</t>
         </is>
       </c>
       <c r="B132" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>$135.49</t>
+          <t>$20.88</t>
         </is>
       </c>
       <c r="D132" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
@@ -4148,23 +4148,23 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>4.64.6 out of 5 stars(173)300+ bought in past month</t>
+          <t>pickleball set with net</t>
         </is>
       </c>
       <c r="B133" s="2" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>$86.99</t>
+          <t>$82.56</t>
         </is>
       </c>
       <c r="D133" s="2" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>48.6%</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
@@ -4176,23 +4176,23 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>52 inch ceiling fan with light and remote white</t>
+          <t>pickleball net portable outdoor</t>
         </is>
       </c>
       <c r="B134" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>$94.67</t>
+          <t>$88.38</t>
         </is>
       </c>
       <c r="D134" s="2" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>40.6%</t>
+          <t>60.6%</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
@@ -4204,23 +4204,23 @@
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>52 inch ceiling fan with light and remote downrod</t>
+          <t>pickleball net outdoor</t>
         </is>
       </c>
       <c r="B135" s="2" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>$95.93</t>
+          <t>$115.31</t>
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>42.4%</t>
+          <t>51.4%</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
@@ -4232,23 +4232,23 @@
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>52 inch ceiling fan with light and remote flush</t>
+          <t>garlic granules 365</t>
         </is>
       </c>
       <c r="B136" s="2" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>$98.67</t>
+          <t>$17.41</t>
         </is>
       </c>
       <c r="D136" s="2" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>63.6%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
@@ -4260,23 +4260,23 @@
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>52 inch ceiling fan no light</t>
+          <t>mjjc foam cannon</t>
         </is>
       </c>
       <c r="B137" s="2" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>$107.57</t>
+          <t>$56.16</t>
         </is>
       </c>
       <c r="D137" s="2" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>40.6%</t>
+          <t>45.5%</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
@@ -4288,23 +4288,23 @@
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>52 inch tv console cabinet</t>
+          <t>baby monitor for car usb c</t>
         </is>
       </c>
       <c r="B138" s="2" t="n">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>$133.41</t>
+          <t>$65.73</t>
         </is>
       </c>
       <c r="D138" s="2" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>48.3%</t>
+          <t>46.7%</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
@@ -4316,23 +4316,23 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>52 inch ceiling fan with light and remote control</t>
+          <t>peelers gummy candy easter</t>
         </is>
       </c>
       <c r="B139" s="2" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>$84.10</t>
+          <t>$20.46</t>
         </is>
       </c>
       <c r="D139" s="2" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>60.6%</t>
+          <t>66.7%</t>
         </is>
       </c>
       <c r="F139" s="2" t="inlineStr">
@@ -4344,23 +4344,23 @@
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>52 inch ceiling fan with led light remote control</t>
+          <t>portable pickleball net</t>
         </is>
       </c>
       <c r="B140" s="2" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>$78.02</t>
+          <t>$118.01</t>
         </is>
       </c>
       <c r="D140" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>59.4%</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr">
@@ -4372,23 +4372,23 @@
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>52 inch ceiling fan with light and remote</t>
+          <t>scotts turf builder rapid grass tall fescue mix - combination grass seed and fertilizer for lawns, lawn seed that grows in just weeks, 5.6 lbs.</t>
         </is>
       </c>
       <c r="B141" s="2" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>$89.41</t>
+          <t>$35.49</t>
         </is>
       </c>
       <c r="D141" s="2" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>79.2%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F141" s="2" t="inlineStr">
@@ -4400,23 +4400,23 @@
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>control pickleball paddles</t>
+          <t>pickleball net set</t>
         </is>
       </c>
       <c r="B142" s="2" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>$83.11</t>
+          <t>$83.02</t>
         </is>
       </c>
       <c r="D142" s="2" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>45.7%</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
@@ -4428,15 +4428,15 @@
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>portable pickleball net with wheels</t>
+          <t>driveway pickleball set with net</t>
         </is>
       </c>
       <c r="B143" s="2" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>$132.37</t>
+          <t>$89.59</t>
         </is>
       </c>
       <c r="D143" s="2" t="n">
@@ -4444,7 +4444,7 @@
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>45.2%</t>
+          <t>42.4%</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
@@ -4456,670 +4456,26 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>wildbird baby carrier plaid</t>
+          <t>oeko-tex standard 100learn more about oeko-tex standard 100</t>
         </is>
       </c>
       <c r="B144" s="2" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>$74.95</t>
+          <t>$48.49</t>
         </is>
       </c>
       <c r="D144" s="2" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>62.5%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="2" t="inlineStr">
-        <is>
-          <t>slk pickleball paddles</t>
-        </is>
-      </c>
-      <c r="B145" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="C145" s="2" t="inlineStr">
-        <is>
-          <t>$89.03</t>
-        </is>
-      </c>
-      <c r="D145" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E145" s="2" t="inlineStr">
-        <is>
-          <t>54.5%</t>
-        </is>
-      </c>
-      <c r="F145" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="2" t="inlineStr">
-        <is>
-          <t>minoxidil foam for women</t>
-        </is>
-      </c>
-      <c r="B146" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="C146" s="2" t="inlineStr">
-        <is>
-          <t>$26.97</t>
-        </is>
-      </c>
-      <c r="D146" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="E146" s="2" t="inlineStr">
-        <is>
-          <t>53.1%</t>
-        </is>
-      </c>
-      <c r="F146" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="2" t="inlineStr">
-        <is>
-          <t>joola pickleball paddle set</t>
-        </is>
-      </c>
-      <c r="B147" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="C147" s="2" t="inlineStr">
-        <is>
-          <t>$103.35</t>
-        </is>
-      </c>
-      <c r="D147" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="E147" s="2" t="inlineStr">
-        <is>
-          <t>45.8%</t>
-        </is>
-      </c>
-      <c r="F147" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="2" t="inlineStr">
-        <is>
-          <t>rogaine 5% minoxidil foam</t>
-        </is>
-      </c>
-      <c r="B148" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="C148" s="2" t="inlineStr">
-        <is>
-          <t>$30.07</t>
-        </is>
-      </c>
-      <c r="D148" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="E148" s="2" t="inlineStr">
-        <is>
-          <t>58.6%</t>
-        </is>
-      </c>
-      <c r="F148" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="2" t="inlineStr">
-        <is>
-          <t>bonide systemic granules for plants</t>
-        </is>
-      </c>
-      <c r="B149" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C149" s="2" t="inlineStr">
-        <is>
-          <t>$20.88</t>
-        </is>
-      </c>
-      <c r="D149" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E149" s="2" t="inlineStr">
-        <is>
-          <t>50.0%</t>
-        </is>
-      </c>
-      <c r="F149" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="2" t="inlineStr">
-        <is>
-          <t>pickleball set with net</t>
-        </is>
-      </c>
-      <c r="B150" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="C150" s="2" t="inlineStr">
-        <is>
-          <t>$82.56</t>
-        </is>
-      </c>
-      <c r="D150" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="E150" s="2" t="inlineStr">
-        <is>
-          <t>48.6%</t>
-        </is>
-      </c>
-      <c r="F150" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="2" t="inlineStr">
-        <is>
-          <t>minoxidil foam for men</t>
-        </is>
-      </c>
-      <c r="B151" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="C151" s="2" t="inlineStr">
-        <is>
-          <t>$28.66</t>
-        </is>
-      </c>
-      <c r="D151" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E151" s="2" t="inlineStr">
-        <is>
-          <t>48.0%</t>
-        </is>
-      </c>
-      <c r="F151" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="2" t="inlineStr">
-        <is>
-          <t>pickleball net portable outdoor</t>
-        </is>
-      </c>
-      <c r="B152" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="C152" s="2" t="inlineStr">
-        <is>
-          <t>$88.38</t>
-        </is>
-      </c>
-      <c r="D152" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="E152" s="2" t="inlineStr">
-        <is>
-          <t>60.6%</t>
-        </is>
-      </c>
-      <c r="F152" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="2" t="inlineStr">
-        <is>
-          <t>pickleball net outdoor</t>
-        </is>
-      </c>
-      <c r="B153" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="C153" s="2" t="inlineStr">
-        <is>
-          <t>$115.31</t>
-        </is>
-      </c>
-      <c r="D153" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="E153" s="2" t="inlineStr">
-        <is>
-          <t>51.4%</t>
-        </is>
-      </c>
-      <c r="F153" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="2" t="inlineStr">
-        <is>
-          <t>garlic granules 365</t>
-        </is>
-      </c>
-      <c r="B154" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="C154" s="2" t="inlineStr">
-        <is>
-          <t>$17.41</t>
-        </is>
-      </c>
-      <c r="D154" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E154" s="2" t="inlineStr">
-        <is>
-          <t>50.0%</t>
-        </is>
-      </c>
-      <c r="F154" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="2" t="inlineStr">
-        <is>
-          <t>mjjc foam cannon</t>
-        </is>
-      </c>
-      <c r="B155" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="C155" s="2" t="inlineStr">
-        <is>
-          <t>$56.16</t>
-        </is>
-      </c>
-      <c r="D155" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E155" s="2" t="inlineStr">
-        <is>
-          <t>45.5%</t>
-        </is>
-      </c>
-      <c r="F155" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="2" t="inlineStr">
-        <is>
-          <t>baby monitor for car usb c</t>
-        </is>
-      </c>
-      <c r="B156" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="C156" s="2" t="inlineStr">
-        <is>
-          <t>$65.73</t>
-        </is>
-      </c>
-      <c r="D156" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="E156" s="2" t="inlineStr">
-        <is>
-          <t>46.7%</t>
-        </is>
-      </c>
-      <c r="F156" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="2" t="inlineStr">
-        <is>
-          <t>minoxidil foam rogaine</t>
-        </is>
-      </c>
-      <c r="B157" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="C157" s="2" t="inlineStr">
-        <is>
-          <t>$30.50</t>
-        </is>
-      </c>
-      <c r="D157" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="E157" s="2" t="inlineStr">
-        <is>
-          <t>57.1%</t>
-        </is>
-      </c>
-      <c r="F157" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="2" t="inlineStr">
-        <is>
-          <t>minoxidil foam</t>
-        </is>
-      </c>
-      <c r="B158" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="C158" s="2" t="inlineStr">
-        <is>
-          <t>$25.22</t>
-        </is>
-      </c>
-      <c r="D158" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="E158" s="2" t="inlineStr">
-        <is>
-          <t>40.0%</t>
-        </is>
-      </c>
-      <c r="F158" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="2" t="inlineStr">
-        <is>
-          <t>peelers gummy candy easter</t>
-        </is>
-      </c>
-      <c r="B159" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="C159" s="2" t="inlineStr">
-        <is>
-          <t>$20.46</t>
-        </is>
-      </c>
-      <c r="D159" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E159" s="2" t="inlineStr">
-        <is>
-          <t>66.7%</t>
-        </is>
-      </c>
-      <c r="F159" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="2" t="inlineStr">
-        <is>
-          <t>minoxidil foam for women hair growth</t>
-        </is>
-      </c>
-      <c r="B160" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="C160" s="2" t="inlineStr">
-        <is>
-          <t>$27.82</t>
-        </is>
-      </c>
-      <c r="D160" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="E160" s="2" t="inlineStr">
-        <is>
-          <t>53.1%</t>
-        </is>
-      </c>
-      <c r="F160" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="2" t="inlineStr">
-        <is>
-          <t>portable pickleball net</t>
-        </is>
-      </c>
-      <c r="B161" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="C161" s="2" t="inlineStr">
-        <is>
-          <t>$118.01</t>
-        </is>
-      </c>
-      <c r="D161" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="E161" s="2" t="inlineStr">
-        <is>
-          <t>59.4%</t>
-        </is>
-      </c>
-      <c r="F161" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="2" t="inlineStr">
-        <is>
-          <t>scotts turf builder rapid grass tall fescue mix - combination grass seed and fertilizer for lawns, lawn seed that grows in just weeks, 5.6 lbs.</t>
-        </is>
-      </c>
-      <c r="B162" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C162" s="2" t="inlineStr">
-        <is>
-          <t>$35.49</t>
-        </is>
-      </c>
-      <c r="D162" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E162" s="2" t="inlineStr">
-        <is>
-          <t>50.0%</t>
-        </is>
-      </c>
-      <c r="F162" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="2" t="inlineStr">
-        <is>
-          <t>pickleball net set</t>
-        </is>
-      </c>
-      <c r="B163" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="C163" s="2" t="inlineStr">
-        <is>
-          <t>$83.02</t>
-        </is>
-      </c>
-      <c r="D163" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="E163" s="2" t="inlineStr">
-        <is>
-          <t>45.7%</t>
-        </is>
-      </c>
-      <c r="F163" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" s="2" t="inlineStr">
-        <is>
-          <t>minoxidil foam kirkland</t>
-        </is>
-      </c>
-      <c r="B164" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="C164" s="2" t="inlineStr">
-        <is>
-          <t>$29.20</t>
-        </is>
-      </c>
-      <c r="D164" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E164" s="2" t="inlineStr">
-        <is>
-          <t>48.0%</t>
-        </is>
-      </c>
-      <c r="F164" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" s="2" t="inlineStr">
-        <is>
-          <t>minoxidil foam 5%</t>
-        </is>
-      </c>
-      <c r="B165" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="C165" s="2" t="inlineStr">
-        <is>
-          <t>$27.11</t>
-        </is>
-      </c>
-      <c r="D165" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E165" s="2" t="inlineStr">
-        <is>
-          <t>40.0%</t>
-        </is>
-      </c>
-      <c r="F165" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="2" t="inlineStr">
-        <is>
-          <t>driveway pickleball set with net</t>
-        </is>
-      </c>
-      <c r="B166" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="C166" s="2" t="inlineStr">
-        <is>
-          <t>$89.59</t>
-        </is>
-      </c>
-      <c r="D166" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="E166" s="2" t="inlineStr">
-        <is>
-          <t>42.4%</t>
-        </is>
-      </c>
-      <c r="F166" s="2" t="inlineStr">
-        <is>
-          <t>✅ GİRİLEBİLİR</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="2" t="inlineStr">
-        <is>
-          <t>oeko-tex standard 100learn more about oeko-tex standard 100</t>
-        </is>
-      </c>
-      <c r="B167" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C167" s="2" t="inlineStr">
-        <is>
-          <t>$48.49</t>
-        </is>
-      </c>
-      <c r="D167" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E167" s="2" t="inlineStr">
-        <is>
-          <t>50.0%</t>
-        </is>
-      </c>
-      <c r="F167" s="2" t="inlineStr">
         <is>
           <t>✅ GİRİLEBİLİR</t>
         </is>

</xml_diff>